<commit_message>
Report charts: show axis labels, single-colour line, currency axis format
</commit_message>
<xml_diff>
--- a/02-excel-report-automation/output/sales_report.xlsx
+++ b/02-excel-report-automation/output/sales_report.xlsx
@@ -177,7 +177,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Monthly revenue</a:t>
+              <a:t>Monthly revenue (USD)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -186,6 +186,7 @@
     <plotArea>
       <lineChart>
         <grouping val="standard"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -217,6 +218,7 @@
               <f>'Monthly'!$D$2:$D$7</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -226,22 +228,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Month</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -252,31 +240,15 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>USD</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -338,6 +310,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -349,16 +322,15 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -420,6 +392,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -431,16 +404,15 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>

</xml_diff>